<commit_message>
Actualizndo concentrado con los datos extraidos de YOLO 	modified:   Seminarios/TablaComparativaConcentrado.xlsx
</commit_message>
<xml_diff>
--- a/Seminarios/TablaComparativaConcentrado.xlsx
+++ b/Seminarios/TablaComparativaConcentrado.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/utrujillo/Documents/Develops/Python/Python3/Vision/analyze_posture_estimation/Seminarios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{345F484D-B5B6-2147-B712-427705AFEF90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00A05C58-A0FC-A54B-B5F8-73E7640D3261}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29500" yWindow="580" windowWidth="10680" windowHeight="16760" activeTab="1" xr2:uid="{0E2D49C4-014D-F645-895F-A57D6B41FEED}"/>
+    <workbookView xWindow="29500" yWindow="580" windowWidth="11720" windowHeight="16760" activeTab="1" xr2:uid="{0E2D49C4-014D-F645-895F-A57D6B41FEED}"/>
   </bookViews>
   <sheets>
     <sheet name="SIV" sheetId="1" r:id="rId1"/>
@@ -87,19 +87,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FFABB2BF"/>
-      <name val="Menlo"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -122,12 +116,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1154,7 +1147,7 @@
       <c r="B20">
         <v>0.1</v>
       </c>
-      <c r="C20" s="2">
+      <c r="C20">
         <v>-38.619799999999998</v>
       </c>
     </row>
@@ -1165,7 +1158,7 @@
       <c r="B21">
         <v>0.5</v>
       </c>
-      <c r="C21" s="2">
+      <c r="C21">
         <v>-38.628799999999998</v>
       </c>
     </row>
@@ -1176,7 +1169,7 @@
       <c r="B22">
         <v>0.9</v>
       </c>
-      <c r="C22" s="2">
+      <c r="C22">
         <v>-38.535899999999998</v>
       </c>
     </row>
@@ -1187,7 +1180,7 @@
       <c r="B23">
         <v>0.1</v>
       </c>
-      <c r="C23" s="2">
+      <c r="C23">
         <v>-9.7489999999999993E-2</v>
       </c>
     </row>
@@ -1198,7 +1191,7 @@
       <c r="B24">
         <v>0.5</v>
       </c>
-      <c r="C24" s="2">
+      <c r="C24">
         <v>-9.7509999999999999E-2</v>
       </c>
     </row>
@@ -1209,7 +1202,7 @@
       <c r="B25">
         <v>0.9</v>
       </c>
-      <c r="C25" s="2">
+      <c r="C25">
         <v>-9.7500000000000003E-2</v>
       </c>
     </row>

</xml_diff>